<commit_message>
updated template with fibo
</commit_message>
<xml_diff>
--- a/files/input/template.xlsx
+++ b/files/input/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ProgramFiles\VM_OS\shared\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0288A32F-502F-46C9-BE70-BA408EE56C81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA8E4CFB-4A90-451E-951E-EC47FB27F444}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="51840" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="31680" yWindow="2880" windowWidth="38700" windowHeight="15375" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -84,7 +84,7 @@
     <t>TitanBot</t>
   </si>
   <si>
-    <t>Fibobot</t>
+    <t>FiboBot</t>
   </si>
 </sst>
 </file>
@@ -196,13 +196,13 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -498,21 +498,21 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{78C930AD-B017-4C45-AEE5-F24DDE5263F9}" name="Table268" displayName="Table268" ref="E83:P89" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="0" tableBorderDxfId="1">
-  <autoFilter ref="E83:P89" xr:uid="{78C930AD-B017-4C45-AEE5-F24DDE5263F9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B0683529-6857-4F8F-87DE-F47B05C4B64B}" name="Table2742" displayName="Table2742" ref="E83:P90" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="0" tableBorderDxfId="1">
+  <autoFilter ref="E83:P90" xr:uid="{B0683529-6857-4F8F-87DE-F47B05C4B64B}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{3A2544FA-2818-4005-8F9E-0316EEF33DD4}" name="trade_id"/>
-    <tableColumn id="2" xr3:uid="{20E8470A-D1B7-49D0-8A65-F566B5AC6868}" name="broker_order_id"/>
-    <tableColumn id="3" xr3:uid="{C45E3CE0-2D0B-4BBD-A90E-BD9E6257FD34}" name="exchange_order_id"/>
-    <tableColumn id="4" xr3:uid="{1384CF59-EE1A-4E07-947A-21E8DB14470E}" name="instrument"/>
-    <tableColumn id="5" xr3:uid="{97CE653F-030A-42A0-B185-C171B8D979A7}" name="instrument_key"/>
-    <tableColumn id="6" xr3:uid="{D4428138-B376-4AF1-BB7D-B70B8A9408A1}" name="side"/>
-    <tableColumn id="7" xr3:uid="{E3C19C5C-EE8F-42E0-9821-679F138A379F}" name="entry"/>
-    <tableColumn id="8" xr3:uid="{363F8B4C-3430-49DF-976F-1A87FF1F014C}" name="exit"/>
-    <tableColumn id="9" xr3:uid="{891B5180-B3BA-433B-94EE-54535269504D}" name="trailed"/>
-    <tableColumn id="10" xr3:uid="{ABEECDDD-FA35-4452-A656-B88CC00F678D}" name="timestamp"/>
-    <tableColumn id="11" xr3:uid="{2706807B-9A28-485B-B2BA-7989F3A30E1F}" name="qty"/>
-    <tableColumn id="12" xr3:uid="{E9ACB2EE-D48E-497C-8025-232002D4420D}" name="amount"/>
+    <tableColumn id="1" xr3:uid="{20CC4563-6EE8-4760-9EF0-26174287EA52}" name="trade_id"/>
+    <tableColumn id="2" xr3:uid="{383DEF5A-47E8-46C7-8488-86C8473C4032}" name="broker_order_id"/>
+    <tableColumn id="3" xr3:uid="{2CC8B1FD-7841-43E0-9E08-A44F4A7852B0}" name="exchange_order_id"/>
+    <tableColumn id="4" xr3:uid="{D247D6E3-0DFE-4F36-854B-92D19A5FE80C}" name="instrument"/>
+    <tableColumn id="5" xr3:uid="{17973419-2332-44E0-8CF4-EDAEE8599B5A}" name="instrument_key"/>
+    <tableColumn id="6" xr3:uid="{F2590BC8-0341-48C7-8A30-23B92C471200}" name="side"/>
+    <tableColumn id="7" xr3:uid="{3F37F559-EC7A-4A80-B33F-6B6723C50F36}" name="entry"/>
+    <tableColumn id="8" xr3:uid="{C1BB9A88-8AE0-48C2-BDE9-C6FA77F41096}" name="exit"/>
+    <tableColumn id="9" xr3:uid="{4B4441DD-CE2C-4CC9-BA11-27FC230AB1C6}" name="trailed"/>
+    <tableColumn id="10" xr3:uid="{35685DD2-8547-4331-980D-994D1BD255FA}" name="timestamp"/>
+    <tableColumn id="11" xr3:uid="{6ABAF89F-7B3D-45D9-83F8-AF2D2DF68AD8}" name="qty"/>
+    <tableColumn id="12" xr3:uid="{00912DE2-5D1E-49AD-AE6C-F04D9D1808AF}" name="amount"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -795,20 +795,20 @@
   </cols>
   <sheetData>
     <row r="3" spans="4:22" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-      <c r="L3" s="8"/>
-      <c r="M3" s="8"/>
-      <c r="N3" s="8"/>
-      <c r="O3" s="8"/>
-      <c r="P3" s="8"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
     </row>
     <row r="4" spans="4:22" x14ac:dyDescent="0.3">
       <c r="D4" s="1"/>
@@ -936,20 +936,20 @@
       <c r="P18" s="7"/>
     </row>
     <row r="22" spans="5:16" x14ac:dyDescent="0.3">
-      <c r="E22" s="6" t="s">
+      <c r="E22" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="6"/>
-      <c r="J22" s="6"/>
-      <c r="K22" s="6"/>
-      <c r="L22" s="6"/>
-      <c r="M22" s="6"/>
-      <c r="N22" s="6"/>
-      <c r="O22" s="6"/>
-      <c r="P22" s="6"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="8"/>
+      <c r="L22" s="8"/>
+      <c r="M22" s="8"/>
+      <c r="N22" s="8"/>
+      <c r="O22" s="8"/>
+      <c r="P22" s="8"/>
     </row>
     <row r="24" spans="5:16" x14ac:dyDescent="0.3">
       <c r="E24" s="2" t="s">
@@ -1056,20 +1056,20 @@
       <c r="P37" s="7"/>
     </row>
     <row r="39" spans="5:16" x14ac:dyDescent="0.3">
-      <c r="E39" s="6" t="s">
+      <c r="E39" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="F39" s="6"/>
-      <c r="G39" s="6"/>
-      <c r="H39" s="6"/>
-      <c r="I39" s="6"/>
-      <c r="J39" s="6"/>
-      <c r="K39" s="6"/>
-      <c r="L39" s="6"/>
-      <c r="M39" s="6"/>
-      <c r="N39" s="6"/>
-      <c r="O39" s="6"/>
-      <c r="P39" s="6"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8"/>
+      <c r="H39" s="8"/>
+      <c r="I39" s="8"/>
+      <c r="J39" s="8"/>
+      <c r="K39" s="8"/>
+      <c r="L39" s="8"/>
+      <c r="M39" s="8"/>
+      <c r="N39" s="8"/>
+      <c r="O39" s="8"/>
+      <c r="P39" s="8"/>
     </row>
     <row r="41" spans="5:16" x14ac:dyDescent="0.3">
       <c r="E41" s="2" t="s">
@@ -1176,20 +1176,20 @@
       <c r="P56" s="7"/>
     </row>
     <row r="60" spans="5:16" x14ac:dyDescent="0.3">
-      <c r="E60" s="6" t="s">
+      <c r="E60" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F60" s="6"/>
-      <c r="G60" s="6"/>
-      <c r="H60" s="6"/>
-      <c r="I60" s="6"/>
-      <c r="J60" s="6"/>
-      <c r="K60" s="6"/>
-      <c r="L60" s="6"/>
-      <c r="M60" s="6"/>
-      <c r="N60" s="6"/>
-      <c r="O60" s="6"/>
-      <c r="P60" s="6"/>
+      <c r="F60" s="8"/>
+      <c r="G60" s="8"/>
+      <c r="H60" s="8"/>
+      <c r="I60" s="8"/>
+      <c r="J60" s="8"/>
+      <c r="K60" s="8"/>
+      <c r="L60" s="8"/>
+      <c r="M60" s="8"/>
+      <c r="N60" s="8"/>
+      <c r="O60" s="8"/>
+      <c r="P60" s="8"/>
     </row>
     <row r="62" spans="5:16" x14ac:dyDescent="0.3">
       <c r="E62" s="2" t="s">
@@ -1295,7 +1295,7 @@
       <c r="O77" s="7"/>
       <c r="P77" s="7"/>
     </row>
-    <row r="81" spans="5:16" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="81" spans="5:16" x14ac:dyDescent="0.3">
       <c r="E81" s="8" t="s">
         <v>19</v>
       </c>
@@ -1310,20 +1310,6 @@
       <c r="N81" s="8"/>
       <c r="O81" s="8"/>
       <c r="P81" s="8"/>
-    </row>
-    <row r="82" spans="5:16" x14ac:dyDescent="0.3">
-      <c r="E82" s="1"/>
-      <c r="F82" s="1"/>
-      <c r="G82" s="1"/>
-      <c r="H82" s="1"/>
-      <c r="I82" s="1"/>
-      <c r="J82" s="1"/>
-      <c r="K82" s="1"/>
-      <c r="L82" s="1"/>
-      <c r="M82" s="1"/>
-      <c r="N82" s="1"/>
-      <c r="O82" s="1"/>
-      <c r="P82" s="1"/>
     </row>
     <row r="83" spans="5:16" x14ac:dyDescent="0.3">
       <c r="E83" s="2" t="s">
@@ -1436,16 +1422,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="E3:P3"/>
+    <mergeCell ref="E15:P18"/>
+    <mergeCell ref="E22:P22"/>
+    <mergeCell ref="E34:P37"/>
     <mergeCell ref="E81:P81"/>
     <mergeCell ref="E93:P96"/>
     <mergeCell ref="E60:P60"/>
     <mergeCell ref="E74:P77"/>
     <mergeCell ref="E39:P39"/>
     <mergeCell ref="E53:P56"/>
-    <mergeCell ref="E3:P3"/>
-    <mergeCell ref="E15:P18"/>
-    <mergeCell ref="E22:P22"/>
-    <mergeCell ref="E34:P37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="5">

</xml_diff>